<commit_message>
UI Fix and the report and function
</commit_message>
<xml_diff>
--- a/test_data/targets_all_branches_may2026.xlsx
+++ b/test_data/targets_all_branches_may2026.xlsx
@@ -1,41 +1,116 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advice\KPV sale performance tracking\test_data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B991FB42-87FA-48E5-895A-AFD4D3D1B2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Targets" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+  <si>
+    <t>Staff_ID</t>
+  </si>
+  <si>
+    <t>Full_Name</t>
+  </si>
+  <si>
+    <t>Branch_ID</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Jewelry_Target_g</t>
+  </si>
+  <si>
+    <t>Bar_Target_g</t>
+  </si>
+  <si>
+    <t>Quantity_Target</t>
+  </si>
+  <si>
+    <t>Somchai Phommachan</t>
+  </si>
+  <si>
+    <t>Khamla Sengdara</t>
+  </si>
+  <si>
+    <t>Boupha Vilayvong</t>
+  </si>
+  <si>
+    <t>Naly Souvannaphoum</t>
+  </si>
+  <si>
+    <t>Daovy Phetchanpheng</t>
+  </si>
+  <si>
+    <t>Savanh Keovongsa</t>
+  </si>
+  <si>
+    <t>Phonesavanh Siha</t>
+  </si>
+  <si>
+    <t>Manivone Keovilay</t>
+  </si>
+  <si>
+    <t>Bounmy Phonsavath</t>
+  </si>
+  <si>
+    <t>Thida Vongsay</t>
+  </si>
+  <si>
+    <t>Khamphone Simoung</t>
+  </si>
+  <si>
+    <t>Soukanh Vongkhamphanh</t>
+  </si>
+  <si>
+    <t>Lattana Phommasack</t>
+  </si>
+  <si>
+    <t>Boualoy Chanthavong</t>
+  </si>
+  <si>
+    <t>Vilasack Keobounma</t>
+  </si>
+  <si>
+    <t>Phouthong Chansouk</t>
+  </si>
+  <si>
+    <t>Souliya Phimmasone</t>
+  </si>
+  <si>
+    <t>Khamsouk Sivilay</t>
+  </si>
+  <si>
+    <t>Nong Phommasith</t>
+  </si>
+  <si>
+    <t>Chanthaly Sitthideth</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +140,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,51 +479,52 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="7.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.09765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Staff_ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Full_Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Branch_ID</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Year</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Month</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Jewelry_Target_g</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Bar_Target_g</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Quantity_Target</v>
-      </c>
-    </row>
-    <row r="2">
+    <row r="1" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="str">
-        <v>Somchai Phommachan</v>
+      <c r="B2" t="s">
+        <v>8</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -461,12 +545,12 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="str">
-        <v>Khamla Sengdara</v>
+      <c r="B3" t="s">
+        <v>9</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -487,12 +571,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="str">
-        <v>Boupha Vilayvong</v>
+      <c r="B4" t="s">
+        <v>10</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -513,12 +597,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="str">
-        <v>Naly Souvannaphoum</v>
+      <c r="B5" t="s">
+        <v>11</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -539,12 +623,12 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="str">
-        <v>Daovy Phetchanpheng</v>
+      <c r="B6" t="s">
+        <v>12</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -565,12 +649,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="str">
-        <v>Savanh Keovongsa</v>
+      <c r="B7" t="s">
+        <v>13</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -591,12 +675,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="str">
-        <v>Phonesavanh Siha</v>
+      <c r="B8" t="s">
+        <v>14</v>
       </c>
       <c r="C8">
         <v>2</v>
@@ -617,12 +701,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="str">
-        <v>Manivone Keovilay</v>
+      <c r="B9" t="s">
+        <v>15</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -643,12 +727,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="str">
-        <v>Bounmy Phonsavath</v>
+      <c r="B10" t="s">
+        <v>16</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -669,12 +753,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="str">
-        <v>Thida Vongsay</v>
+      <c r="B11" t="s">
+        <v>17</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -695,12 +779,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="str">
-        <v>Khamphone Simoung</v>
+      <c r="B12" t="s">
+        <v>18</v>
       </c>
       <c r="C12">
         <v>3</v>
@@ -721,12 +805,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" t="str">
-        <v>Soukanh Vongkhamphanh</v>
+      <c r="B13" t="s">
+        <v>19</v>
       </c>
       <c r="C13">
         <v>3</v>
@@ -747,12 +831,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" t="str">
-        <v>Lattana Phommasack</v>
+      <c r="B14" t="s">
+        <v>20</v>
       </c>
       <c r="C14">
         <v>3</v>
@@ -773,12 +857,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" t="str">
-        <v>Boualoy Chanthavong</v>
+      <c r="B15" t="s">
+        <v>21</v>
       </c>
       <c r="C15">
         <v>3</v>
@@ -799,12 +883,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" t="str">
-        <v>Vilasack Keobounma</v>
+      <c r="B16" t="s">
+        <v>22</v>
       </c>
       <c r="C16">
         <v>3</v>
@@ -825,12 +909,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" t="str">
-        <v>Phouthong Chansouk</v>
+      <c r="B17" t="s">
+        <v>23</v>
       </c>
       <c r="C17">
         <v>4</v>
@@ -851,12 +935,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" t="str">
-        <v>Souliya Phimmasone</v>
+      <c r="B18" t="s">
+        <v>24</v>
       </c>
       <c r="C18">
         <v>4</v>
@@ -877,12 +961,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" t="str">
-        <v>Khamsouk Sivilay</v>
+      <c r="B19" t="s">
+        <v>25</v>
       </c>
       <c r="C19">
         <v>4</v>
@@ -903,12 +987,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" t="str">
-        <v>Nong Phommasith</v>
+      <c r="B20" t="s">
+        <v>26</v>
       </c>
       <c r="C20">
         <v>4</v>
@@ -929,12 +1013,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" t="str">
-        <v>Chanthaly Sitthideth</v>
+      <c r="B21" t="s">
+        <v>27</v>
       </c>
       <c r="C21">
         <v>4</v>
@@ -956,8 +1040,9 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
+    <ignoredError sqref="A1:H21" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>